<commit_message>
2026.05.16 Test Change 38.
</commit_message>
<xml_diff>
--- a/git環境の構築手順.xlsx
+++ b/git環境の構築手順.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\WORK\git-repositories\test_20260426\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F617CE4F-A72D-4862-A324-17FA822F711B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E545808D-5883-40C8-8076-CF56D69AA560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1905" yWindow="1605" windowWidth="23100" windowHeight="18735" xr2:uid="{60E057AB-4F0C-4147-97E2-0AB2076230C2}"/>
+    <workbookView xWindow="1905" yWindow="1605" windowWidth="29100" windowHeight="18735" activeTab="1" xr2:uid="{60E057AB-4F0C-4147-97E2-0AB2076230C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Git環境について" sheetId="1" r:id="rId1"/>
+    <sheet name="GitのHEADとは何者なのか" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1204,6 +1205,668 @@
         <a:xfrm>
           <a:off x="7181850" y="38423850"/>
           <a:ext cx="6887536" cy="4838700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>601116</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>220103</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="図 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AFEDFB64-3354-2220-C7F2-91CEC0CDF630}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7459116" cy="7363853"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>220063</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>1230</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="図 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{28DAD56D-FB19-990A-D757-F950F9C0D1FA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="7620000"/>
+          <a:ext cx="7078063" cy="8811855"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>439168</xdr:colOff>
+      <xdr:row>104</xdr:row>
+      <xdr:rowOff>125006</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="図 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3DB492F4-E11F-836D-EA6D-F42E77053BB6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="16430625"/>
+          <a:ext cx="7297168" cy="8459381"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>105</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>534432</xdr:colOff>
+      <xdr:row>146</xdr:row>
+      <xdr:rowOff>201416</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="図 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1ED01C7-76B7-BCBF-95E2-920667293394}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="25003125"/>
+          <a:ext cx="7392432" cy="9964541"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>148</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>181957</xdr:colOff>
+      <xdr:row>185</xdr:row>
+      <xdr:rowOff>191756</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="図 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6B0847B6-7473-0700-AFFA-435449500CEF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="35242500"/>
+          <a:ext cx="7039957" cy="9002381"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>186</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>20010</xdr:colOff>
+      <xdr:row>192</xdr:row>
+      <xdr:rowOff>181200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="図 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ACADA372-D3EC-51A6-0ACB-AEB9BDAA9CBA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="44291250"/>
+          <a:ext cx="6878010" cy="1609950"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>685799</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>676274</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>220568</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="図 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{04F555F7-2968-39F2-E185-14F26EABBF24}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8229599" y="0"/>
+          <a:ext cx="6848475" cy="10698068"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>9524</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>143403</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="15" name="グループ化 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D4111DDC-3269-66B1-89CD-A81BB040258F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="8239124" y="10648950"/>
+          <a:ext cx="6886576" cy="3781953"/>
+          <a:chOff x="8239124" y="10648950"/>
+          <a:chExt cx="6886576" cy="3781953"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="10" name="図 9">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AF15305A-0347-6DEE-5527-7882D601832D}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8239124" y="10648950"/>
+            <a:ext cx="6886576" cy="3781953"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="11" name="正方形/長方形 10">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9793D40B-1438-306B-2BEB-9CA9FC9A8668}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8477250" y="12658724"/>
+            <a:ext cx="4267200" cy="209551"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="25400">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr kumimoji="1" lang="ja-JP" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="12" name="正方形/長方形 11">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A366A3D7-9DD3-7258-505C-4B3554676B62}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8963024" y="11191875"/>
+            <a:ext cx="4733925" cy="219076"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="25400">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr kumimoji="1" lang="ja-JP" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="14" name="正方形/長方形 13">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4346C281-D212-D289-B466-B3BCB455C56C}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="9077324" y="11753849"/>
+            <a:ext cx="4695825" cy="228601"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="25400">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr kumimoji="1" lang="ja-JP" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>219075</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>88</xdr:row>
+      <xdr:rowOff>229499</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="図 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3168BFEC-1368-5A6A-D5CF-14EDB2780E85}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8277225" y="14744700"/>
+          <a:ext cx="7086600" cy="6439799"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>128</xdr:row>
+      <xdr:rowOff>29842</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="図 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9A9FC85-D6B9-A525-C5CB-0EA4D789D987}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8229600" y="21431250"/>
+          <a:ext cx="6991350" cy="9078592"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>129</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>333375</xdr:colOff>
+      <xdr:row>159</xdr:row>
+      <xdr:rowOff>67681</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="図 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12C08434-1C1F-0A8C-0074-0CE15F3E89E0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8229600" y="30718125"/>
+          <a:ext cx="7191375" cy="7211431"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2793,4 +3456,15 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C83F0D9-DE33-4E6B-BABB-40422D193EEA}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetData/>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
2026.05.16 Test Change 37.
</commit_message>
<xml_diff>
--- a/git環境の構築手順.xlsx
+++ b/git環境の構築手順.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\WORK\git-repositories\test_20260426\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F617CE4F-A72D-4862-A324-17FA822F711B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E545808D-5883-40C8-8076-CF56D69AA560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1905" yWindow="1605" windowWidth="23100" windowHeight="18735" xr2:uid="{60E057AB-4F0C-4147-97E2-0AB2076230C2}"/>
+    <workbookView xWindow="1905" yWindow="1605" windowWidth="29100" windowHeight="18735" activeTab="1" xr2:uid="{60E057AB-4F0C-4147-97E2-0AB2076230C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Git環境について" sheetId="1" r:id="rId1"/>
+    <sheet name="GitのHEADとは何者なのか" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1204,6 +1205,668 @@
         <a:xfrm>
           <a:off x="7181850" y="38423850"/>
           <a:ext cx="6887536" cy="4838700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>601116</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>220103</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="図 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AFEDFB64-3354-2220-C7F2-91CEC0CDF630}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7459116" cy="7363853"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>220063</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>1230</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="図 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{28DAD56D-FB19-990A-D757-F950F9C0D1FA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="7620000"/>
+          <a:ext cx="7078063" cy="8811855"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>439168</xdr:colOff>
+      <xdr:row>104</xdr:row>
+      <xdr:rowOff>125006</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="図 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3DB492F4-E11F-836D-EA6D-F42E77053BB6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="16430625"/>
+          <a:ext cx="7297168" cy="8459381"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>105</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>534432</xdr:colOff>
+      <xdr:row>146</xdr:row>
+      <xdr:rowOff>201416</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="図 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1ED01C7-76B7-BCBF-95E2-920667293394}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="25003125"/>
+          <a:ext cx="7392432" cy="9964541"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>148</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>181957</xdr:colOff>
+      <xdr:row>185</xdr:row>
+      <xdr:rowOff>191756</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="図 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6B0847B6-7473-0700-AFFA-435449500CEF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="35242500"/>
+          <a:ext cx="7039957" cy="9002381"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>186</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>20010</xdr:colOff>
+      <xdr:row>192</xdr:row>
+      <xdr:rowOff>181200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="図 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ACADA372-D3EC-51A6-0ACB-AEB9BDAA9CBA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="44291250"/>
+          <a:ext cx="6878010" cy="1609950"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>685799</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>676274</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>220568</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="図 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{04F555F7-2968-39F2-E185-14F26EABBF24}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8229599" y="0"/>
+          <a:ext cx="6848475" cy="10698068"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>9524</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>143403</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="15" name="グループ化 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D4111DDC-3269-66B1-89CD-A81BB040258F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="8239124" y="10648950"/>
+          <a:ext cx="6886576" cy="3781953"/>
+          <a:chOff x="8239124" y="10648950"/>
+          <a:chExt cx="6886576" cy="3781953"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="10" name="図 9">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AF15305A-0347-6DEE-5527-7882D601832D}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8239124" y="10648950"/>
+            <a:ext cx="6886576" cy="3781953"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="11" name="正方形/長方形 10">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9793D40B-1438-306B-2BEB-9CA9FC9A8668}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8477250" y="12658724"/>
+            <a:ext cx="4267200" cy="209551"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="25400">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr kumimoji="1" lang="ja-JP" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="12" name="正方形/長方形 11">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A366A3D7-9DD3-7258-505C-4B3554676B62}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8963024" y="11191875"/>
+            <a:ext cx="4733925" cy="219076"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="25400">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr kumimoji="1" lang="ja-JP" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="14" name="正方形/長方形 13">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4346C281-D212-D289-B466-B3BCB455C56C}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="9077324" y="11753849"/>
+            <a:ext cx="4695825" cy="228601"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="25400">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr kumimoji="1" lang="ja-JP" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>219075</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>88</xdr:row>
+      <xdr:rowOff>229499</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="図 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3168BFEC-1368-5A6A-D5CF-14EDB2780E85}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8277225" y="14744700"/>
+          <a:ext cx="7086600" cy="6439799"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>128</xdr:row>
+      <xdr:rowOff>29842</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="図 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9A9FC85-D6B9-A525-C5CB-0EA4D789D987}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8229600" y="21431250"/>
+          <a:ext cx="6991350" cy="9078592"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>129</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>333375</xdr:colOff>
+      <xdr:row>159</xdr:row>
+      <xdr:rowOff>67681</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="図 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12C08434-1C1F-0A8C-0074-0CE15F3E89E0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8229600" y="30718125"/>
+          <a:ext cx="7191375" cy="7211431"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2793,4 +3456,15 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C83F0D9-DE33-4E6B-BABB-40422D193EEA}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetData/>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>